<commit_message>
docs: add sms pending cost, steel instructions, tom losito template
</commit_message>
<xml_diff>
--- a/products/steel-estimator/Steel_Estimator_CSI_MasterFormat.xlsx
+++ b/products/steel-estimator/Steel_Estimator_CSI_MasterFormat.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-Project Setup" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-Fabrication" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-Project Setup" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-Erection" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4-Summary" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
@@ -474,6 +474,70 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Steel Estimator – Instructions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. Complete the data entry on Sheet 1 (Project Setup).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2. Fabrication (Sheet 2) and Erection (Sheet 3) are pre-coded with CSI Division 05 items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3. Update QTY / Crew / Hrs-Unit columns only; CSI Code/Line IDs stay locked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4. Summary (Sheet 4) auto-calculates totals by CSI code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5. Use the drop-down at the top of each sheet to toggle GC vs. Sub view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6. Duplicate this workbook per project and archive a clean master copy.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -843,1433 +907,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A15:F15"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A15:F15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FABRICATION ESTIMATE - CSI DIVISION 05: METALS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>CSI Division: 05 | CSI Code: 05 10 00 | Description: Structural Metal Framing</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Line</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>CSI Code</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Item Description</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Spec/Material</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Material $/Unit</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>Material Cost</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr">
-        <is>
-          <t>Fab Hours</t>
-        </is>
-      </c>
-      <c r="L4" s="8" t="inlineStr">
-        <is>
-          <t>Labor Rate</t>
-        </is>
-      </c>
-      <c r="M4" s="8" t="inlineStr">
-        <is>
-          <t>Labor Cost</t>
-        </is>
-      </c>
-      <c r="N4" s="8" t="inlineStr">
-        <is>
-          <t>Subtotal</t>
-        </is>
-      </c>
-      <c r="O4" s="8" t="inlineStr">
-        <is>
-          <t>Markup %</t>
-        </is>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>F-001</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>STRUCTURAL BEAMS</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>W36x300 Beams</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n">
-        <v>300</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="J5" s="9">
-        <f>G5*I5</f>
-        <v/>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M5" s="9">
-        <f>K5*L5</f>
-        <v/>
-      </c>
-      <c r="N5" s="9">
-        <f>J5+M5</f>
-        <v/>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P5" s="9">
-        <f>N5*(1+O5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>F-002</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>W36x230 Beams</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n">
-        <v>230</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>3.85</v>
-      </c>
-      <c r="J6" s="9">
-        <f>G6*I6</f>
-        <v/>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M6" s="9">
-        <f>K6*L6</f>
-        <v/>
-      </c>
-      <c r="N6" s="9">
-        <f>J6+M6</f>
-        <v/>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P6" s="9">
-        <f>N6*(1+O6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>F-003</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>W33x241 Beams</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n">
-        <v>241</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>3.65</v>
-      </c>
-      <c r="J7" s="9">
-        <f>G7*I7</f>
-        <v/>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="L7" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M7" s="9">
-        <f>K7*L7</f>
-        <v/>
-      </c>
-      <c r="N7" s="9">
-        <f>J7+M7</f>
-        <v/>
-      </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P7" s="9">
-        <f>N7*(1+O7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>F-004</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>W30x211 Beams</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n">
-        <v>211</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="J8" s="9">
-        <f>G8*I8</f>
-        <v/>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M8" s="9">
-        <f>K8*L8</f>
-        <v/>
-      </c>
-      <c r="N8" s="9">
-        <f>J8+M8</f>
-        <v/>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P8" s="9">
-        <f>N8*(1+O8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>F-005</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>W27x194 Beams</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n">
-        <v>194</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="J9" s="9">
-        <f>G9*I9</f>
-        <v/>
-      </c>
-      <c r="K9" s="5" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="L9" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M9" s="9">
-        <f>K9*L9</f>
-        <v/>
-      </c>
-      <c r="N9" s="9">
-        <f>J9+M9</f>
-        <v/>
-      </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P9" s="9">
-        <f>N9*(1+O9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>F-006</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>W24x162 Beams</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n">
-        <v>162</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="J10" s="9">
-        <f>G10*I10</f>
-        <v/>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M10" s="9">
-        <f>K10*L10</f>
-        <v/>
-      </c>
-      <c r="N10" s="9">
-        <f>J10+M10</f>
-        <v/>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P10" s="9">
-        <f>N10*(1+O10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>F-007</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>W21x147 Beams</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n">
-        <v>147</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>2.85</v>
-      </c>
-      <c r="J11" s="9">
-        <f>G11*I11</f>
-        <v/>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L11" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M11" s="9">
-        <f>K11*L11</f>
-        <v/>
-      </c>
-      <c r="N11" s="9">
-        <f>J11+M11</f>
-        <v/>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P11" s="9">
-        <f>N11*(1+O11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>F-008</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>W18x119 Beams</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n">
-        <v>119</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="J12" s="9">
-        <f>G12*I12</f>
-        <v/>
-      </c>
-      <c r="K12" s="5" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="L12" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M12" s="9">
-        <f>K12*L12</f>
-        <v/>
-      </c>
-      <c r="N12" s="9">
-        <f>J12+M12</f>
-        <v/>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P12" s="9">
-        <f>N12*(1+O12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>F-009</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.19</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>W16x100 Beams</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>2.45</v>
-      </c>
-      <c r="J13" s="9">
-        <f>G13*I13</f>
-        <v/>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="L13" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M13" s="9">
-        <f>K13*L13</f>
-        <v/>
-      </c>
-      <c r="N13" s="9">
-        <f>J13+M13</f>
-        <v/>
-      </c>
-      <c r="O13" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P13" s="9">
-        <f>N13*(1+O13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>F-010</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.23</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>STRUCTURAL COLUMNS</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>W14x90 Columns</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="I14" s="5" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="J14" s="9">
-        <f>G14*I14</f>
-        <v/>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="L14" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M14" s="9">
-        <f>K14*L14</f>
-        <v/>
-      </c>
-      <c r="N14" s="9">
-        <f>J14+M14</f>
-        <v/>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P14" s="9">
-        <f>N14*(1+O14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>F-011</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.23</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr"/>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>W12x65 Columns</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n">
-        <v>65</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="J15" s="9">
-        <f>G15*I15</f>
-        <v/>
-      </c>
-      <c r="K15" s="5" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="L15" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M15" s="9">
-        <f>K15*L15</f>
-        <v/>
-      </c>
-      <c r="N15" s="9">
-        <f>J15+M15</f>
-        <v/>
-      </c>
-      <c r="O15" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P15" s="9">
-        <f>N15*(1+O15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>F-012</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>05 10 13.23</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>W10x49 Columns</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>A992 Gr50</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n">
-        <v>49</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>1.85</v>
-      </c>
-      <c r="J16" s="9">
-        <f>G16*I16</f>
-        <v/>
-      </c>
-      <c r="K16" s="5" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="L16" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M16" s="9">
-        <f>K16*L16</f>
-        <v/>
-      </c>
-      <c r="N16" s="9">
-        <f>J16+M16</f>
-        <v/>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P16" s="9">
-        <f>N16*(1+O16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>F-013</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>05 20 00</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>METAL JOISTS</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>K-Series Joists</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>ASTM A572</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="I17" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="J17" s="9">
-        <f>G17*I17</f>
-        <v/>
-      </c>
-      <c r="K17" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="L17" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M17" s="9">
-        <f>K17*L17</f>
-        <v/>
-      </c>
-      <c r="N17" s="9">
-        <f>J17+M17</f>
-        <v/>
-      </c>
-      <c r="O17" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P17" s="9">
-        <f>N17*(1+O17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>F-014</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>05 20 00</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>LH-Series Joists</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>ASTM A572</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="J18" s="9">
-        <f>G18*I18</f>
-        <v/>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="L18" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M18" s="9">
-        <f>K18*L18</f>
-        <v/>
-      </c>
-      <c r="N18" s="9">
-        <f>J18+M18</f>
-        <v/>
-      </c>
-      <c r="O18" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P18" s="9">
-        <f>N18*(1+O18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>F-015</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>05 30 00</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>METAL DECKING</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>1.5" B-Deck</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>G60 Galv</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="J19" s="9">
-        <f>G19*I19</f>
-        <v/>
-      </c>
-      <c r="K19" s="5" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="L19" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M19" s="9">
-        <f>K19*L19</f>
-        <v/>
-      </c>
-      <c r="N19" s="9">
-        <f>J19+M19</f>
-        <v/>
-      </c>
-      <c r="O19" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P19" s="9">
-        <f>N19*(1+O19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>F-016</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>05 30 00</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>3.0" N-Deck</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>G60 Galv</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>SF</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="J20" s="9">
-        <f>G20*I20</f>
-        <v/>
-      </c>
-      <c r="K20" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="L20" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M20" s="9">
-        <f>K20*L20</f>
-        <v/>
-      </c>
-      <c r="N20" s="9">
-        <f>J20+M20</f>
-        <v/>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P20" s="9">
-        <f>N20*(1+O20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>F-017</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>05 40 00</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>COLD-FORMED FRAMING</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>C-Studs 6"</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>G90 Galv</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="J21" s="9">
-        <f>G21*I21</f>
-        <v/>
-      </c>
-      <c r="K21" s="5" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="L21" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M21" s="9">
-        <f>K21*L21</f>
-        <v/>
-      </c>
-      <c r="N21" s="9">
-        <f>J21+M21</f>
-        <v/>
-      </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P21" s="9">
-        <f>N21*(1+O21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>F-018</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>05 50 00</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>METAL FABRICATIONS</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Stairs &amp; Railings</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>A500 Gr B</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>LS</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="I22" s="5" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J22" s="9">
-        <f>G22*I22</f>
-        <v/>
-      </c>
-      <c r="K22" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="L22" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M22" s="9">
-        <f>K22*L22</f>
-        <v/>
-      </c>
-      <c r="N22" s="9">
-        <f>J22+M22</f>
-        <v/>
-      </c>
-      <c r="O22" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P22" s="9">
-        <f>N22*(1+O22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>F-019</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>05 50 00</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Ladders</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>A500 Gr B</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n">
-        <v>450</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <v>450</v>
-      </c>
-      <c r="J23" s="9">
-        <f>G23*I23</f>
-        <v/>
-      </c>
-      <c r="K23" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="L23" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M23" s="9">
-        <f>K23*L23</f>
-        <v/>
-      </c>
-      <c r="N23" s="9">
-        <f>J23+M23</f>
-        <v/>
-      </c>
-      <c r="O23" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P23" s="9">
-        <f>N23*(1+O23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>F-020</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>05 70 00</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>ORNAMENTAL METAL</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Decorative Railings</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Aluminum</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>LF</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n">
-        <v>85</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <v>85</v>
-      </c>
-      <c r="J24" s="9">
-        <f>G24*I24</f>
-        <v/>
-      </c>
-      <c r="K24" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="L24" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="M24" s="9">
-        <f>K24*L24</f>
-        <v/>
-      </c>
-      <c r="N24" s="9">
-        <f>J24+M24</f>
-        <v/>
-      </c>
-      <c r="O24" s="5" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="P24" s="9">
-        <f>N24*(1+O24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>FABRICATION TOTALS</t>
-        </is>
-      </c>
-      <c r="J26" s="10">
-        <f>SUM(J5:J24)</f>
-        <v/>
-      </c>
-      <c r="M26" s="10">
-        <f>SUM(M5:M24)</f>
-        <v/>
-      </c>
-      <c r="N26" s="10">
-        <f>SUM(N5:N24)</f>
-        <v/>
-      </c>
-      <c r="P26" s="10">
-        <f>SUM(P5:P24)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3601,8 +2240,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="A2:N2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3663,7 +2302,6 @@
           <t>Project Name:</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3671,7 +2309,6 @@
           <t>Project Number:</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3679,7 +2316,6 @@
           <t>Client:</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3687,7 +2323,6 @@
           <t>Location:</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3695,7 +2330,6 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3703,7 +2337,6 @@
           <t>Estimator:</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4155,11 +2788,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A14:D14"/>
-    <mergeCell ref="A28:C28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>